<commit_message>
add production reporting and fastener validation
</commit_message>
<xml_diff>
--- a/数据层.xlsx
+++ b/数据层.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\work\studyAndLearn\SWApiDesign\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E4F946-3EFB-402B-876C-9346DDF563C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C303AFF-F439-4AF6-B171-2708AB58201A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2745" yWindow="2745" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="152">
   <si>
     <t>配电箱铜排连接系统 · 二次开发数据层模板</t>
   </si>
@@ -506,6 +506,14 @@
   </si>
   <si>
     <t>M16</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>平垫直径</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>螺栓头直径</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -694,12 +702,12 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1014,7 +1022,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="15"/>
@@ -1096,7 +1104,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="15"/>
@@ -1113,7 +1121,7 @@
       <c r="M1" s="15"/>
     </row>
     <row r="2" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="15"/>
@@ -1792,10 +1800,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED5DC8E-8DC7-4888-8A45-566AC4631725}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.15">
       <c r="A1" s="3" t="s">
         <v>25</v>
       </c>
@@ -1821,13 +1832,19 @@
         <v>142</v>
       </c>
       <c r="I1" t="s">
+        <v>150</v>
+      </c>
+      <c r="J1" t="s">
         <v>143</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="L1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>145</v>
       </c>
@@ -1847,13 +1864,19 @@
         <v>1.5</v>
       </c>
       <c r="I2">
+        <v>16</v>
+      </c>
+      <c r="J2">
         <v>6</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="L2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>146</v>
       </c>
@@ -1879,13 +1902,19 @@
         <v>2</v>
       </c>
       <c r="I3">
+        <v>20</v>
+      </c>
+      <c r="J3">
         <v>8</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="L3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>147</v>
       </c>
@@ -1908,13 +1937,19 @@
         <v>2.5</v>
       </c>
       <c r="I4">
+        <v>24</v>
+      </c>
+      <c r="J4">
         <v>11</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="L4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>148</v>
       </c>
@@ -1934,13 +1969,19 @@
         <v>2.5</v>
       </c>
       <c r="I5">
+        <v>28</v>
+      </c>
+      <c r="J5">
         <v>11</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>9.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="L5">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
         <v>149</v>
       </c>
@@ -1960,10 +2001,16 @@
         <v>3</v>
       </c>
       <c r="I6">
+        <v>32</v>
+      </c>
+      <c r="J6">
         <v>14</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>11</v>
+      </c>
+      <c r="L6">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1991,7 +2038,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>51</v>
       </c>
       <c r="B1" s="15"/>
@@ -2007,7 +2054,7 @@
       <c r="L1" s="15"/>
     </row>
     <row r="2" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="15"/>
@@ -2071,7 +2118,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="6">
-        <f t="shared" ref="D4:D12" si="0">B4*C4</f>
+        <f t="shared" ref="D4:D11" si="0">B4*C4</f>
         <v>120</v>
       </c>
       <c r="E4" s="6"/>
@@ -2286,7 +2333,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>70</v>
       </c>
       <c r="B1" s="15"/>
@@ -2298,7 +2345,7 @@
       <c r="H1" s="15"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>71</v>
       </c>
       <c r="B2" s="15"/>
@@ -2476,7 +2523,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>86</v>
       </c>
       <c r="B1" s="15"/>

</xml_diff>